<commit_message>
Version 2: one entry per dog, personalised emails, save progress
- Allow one row per dog; never match an account to itself; all rows for
  an account must share country and Will Send To
- Avoid one account sending to the same account twice, then swaps,
  unless there is no other way (faster incremental search)
- <Your Dog's Name> marker for the greeting and subject; per-entry
  spending wording
- Save progress button and reminder every 10 ticks; Gmail reuses one tab
- Summarised impossible-draw explanations with folded name lists
- Master list records the giver's dog; reload by account and dog
- Updated test spreadsheet, trial instructions (with Mac steps) and plan

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DD7WxN7dAAyJNhu4kdPm7N
</commit_message>
<xml_diff>
--- a/test-dummy.xlsx
+++ b/test-dummy.xlsx
@@ -413,11 +413,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F81"/>
+  <dimension ref="A1:F79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="60" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
@@ -464,7 +464,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Bramble</t>
+          <t>Fudge</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -479,7 +479,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Any</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -496,7 +496,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Daisy &amp; Biscuit</t>
+          <t>Murphy</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -511,7 +511,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Any</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -528,7 +528,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Daisy</t>
+          <t>Clover</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -543,7 +543,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Any</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -560,7 +560,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Rolo</t>
+          <t>Juniper</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -592,7 +592,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Rolo</t>
+          <t>Ziggy</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -607,7 +607,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Any</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -656,7 +656,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Daisy</t>
+          <t>Pippin</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -688,7 +688,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Luna &amp; Pippin</t>
+          <t>Daisy</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -720,7 +720,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Pippin</t>
+          <t>Archie</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -752,7 +752,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Mabel &amp; Otis</t>
+          <t>Ziggy</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -767,7 +767,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Any</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -784,7 +784,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Rolo</t>
+          <t>Ziggy</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -816,7 +816,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Tilly</t>
+          <t>Juniper</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -848,7 +848,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Bramble</t>
+          <t>Daisy</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -863,7 +863,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>Any</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -880,7 +880,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Nell</t>
+          <t>Luna</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -895,7 +895,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>Any</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -912,7 +912,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Luna &amp; Willow</t>
+          <t>Murphy</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -944,7 +944,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Bramble</t>
+          <t>Clover</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -976,7 +976,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Rolo &amp; Poppy</t>
+          <t>Juniper</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -991,7 +991,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Any</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1008,7 +1008,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Bramble</t>
+          <t>Willow</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1023,7 +1023,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>Any</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1040,7 +1040,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Daisy</t>
+          <t>Rolo</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1055,7 +1055,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Any</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1072,7 +1072,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Bramble</t>
+          <t>Hector</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1087,7 +1087,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Any</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1104,7 +1104,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Tilly</t>
+          <t>Fudge</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>Any</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1168,7 +1168,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Rolo &amp; Willow</t>
+          <t>Bramble</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1200,7 +1200,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Murphy</t>
+          <t>Juniper</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1215,7 +1215,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Any</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1232,7 +1232,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Nell &amp; Murphy</t>
+          <t>Rolo</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1279,7 +1279,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Any</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1296,7 +1296,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Willow &amp; Luna</t>
+          <t>Willow</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1328,7 +1328,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Tilly &amp; Murphy</t>
+          <t>Bertie</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1360,7 +1360,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Hector</t>
+          <t>Bertie</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1392,7 +1392,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Hector</t>
+          <t>Daisy</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1407,7 +1407,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>Any</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Any</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1456,7 +1456,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Mabel</t>
+          <t>Clover</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1471,7 +1471,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>Any</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1488,7 +1488,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Bertie</t>
+          <t>Hector</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1520,7 +1520,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Hector</t>
+          <t>Willow</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1552,7 +1552,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Nell</t>
+          <t>Poppy</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1584,7 +1584,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Pippin</t>
+          <t>Biscuit</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1616,7 +1616,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Daisy</t>
+          <t>Biscuit</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1631,7 +1631,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>Any</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -1643,17 +1643,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>test_dog_38</t>
+          <t>test_dog_37</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Archie</t>
+          <t>Bertie</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Owner 38, 38 Test Street, Anytown, AB1 2CD, UK</t>
+          <t>Owner 37, 37 Test Street, Anytown, AB1 2CD, UK</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1668,14 +1668,14 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>test_dog_38@example.com</t>
+          <t>test_dog_37@example.com</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>test_dog_39</t>
+          <t>test_dog_38</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1685,7 +1685,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Owner 39, 39 Test Street, Anytown, AB1 2CD, UK</t>
+          <t>Owner 38, 38 Test Street, Anytown, AB1 2CD, UK</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1700,24 +1700,24 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>test_dog_39@example.com</t>
+          <t>test_dog_38@example.com</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>test_dog_40</t>
+          <t>test_dog_38</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Rolo</t>
+          <t>Mabel</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Owner 40, 40 Test Street, Anytown, AB1 2CD, UK</t>
+          <t>Owner 38, 38 Test Street, Anytown, AB1 2CD, UK</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1732,24 +1732,24 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>test_dog_40@example.com</t>
+          <t>test_dog_38@example.com</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>test_dog_41</t>
+          <t>test_dog_39</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Biscuit</t>
+          <t>Otis</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Owner 41, 41 Test Street, Anytown, AB1 2CD, UK</t>
+          <t>Owner 39, 39 Test Street, Anytown, AB1 2CD, UK</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1759,29 +1759,29 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Any</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>test_dog_41@example.com</t>
+          <t>test_dog_39@example.com</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>test_dog_42</t>
+          <t>test_dog_39</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Bertie</t>
+          <t>Murphy</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Owner 42, 42 Test Street, Anytown, AB1 2CD, UK</t>
+          <t>Owner 39, 39 Test Street, Anytown, AB1 2CD, UK</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1796,24 +1796,24 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>test_dog_42@example.com</t>
+          <t>test_dog_39@example.com</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>test_dog_43</t>
+          <t>test_dog_40</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Nell</t>
+          <t>Pippin</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Owner 43, 43 Test Street, Springfield, OH, 45501, USA</t>
+          <t>Owner 40, 40 Test Street, Springfield, OH, 45501, USA</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1823,29 +1823,29 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Any</t>
+          <t>Canada, USA</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>test_dog_43@example.com</t>
+          <t>test_dog_40@example.com</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>test_dog_44</t>
+          <t>test_dog_41</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Otis</t>
+          <t>Archie</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Owner 44, 44 Test Street, Springfield, OH, 45501, USA</t>
+          <t>Owner 41, 41 Test Street, Springfield, OH, 45501, USA</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1860,24 +1860,24 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>test_dog_44@example.com</t>
+          <t>test_dog_41@example.com</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>test_dog_45</t>
+          <t>test_dog_42</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Hector</t>
+          <t>Poppy</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Owner 45, 45 Test Street, Springfield, OH, 45501, USA</t>
+          <t>Owner 42, 42 Test Street, Springfield, OH, 45501, USA</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -1887,29 +1887,29 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Canada, USA</t>
+          <t>Any</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>test_dog_45@example.com</t>
+          <t>test_dog_42@example.com</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>test_dog_46</t>
+          <t>test_dog_43</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Tilly &amp; Tilly</t>
+          <t>Bertie</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Owner 46, 46 Test Street, Springfield, OH, 45501, USA</t>
+          <t>Owner 43, 43 Test Street, Springfield, OH, 45501, USA</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -1924,24 +1924,24 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>test_dog_46@example.com</t>
+          <t>test_dog_43@example.com</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>test_dog_47</t>
+          <t>test_dog_44</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Murphy</t>
+          <t>Clover</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Owner 47, 47 Test Street, Springfield, OH, 45501, USA</t>
+          <t>Owner 44, 44 Test Street, Springfield, OH, 45501, USA</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -1956,24 +1956,24 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>test_dog_47@example.com</t>
+          <t>test_dog_44@example.com</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>test_dog_48</t>
+          <t>test_dog_45</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Pippin &amp; Bramble</t>
+          <t>Bertie</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Owner 48, 48 Test Street, Springfield, OH, 45501, USA</t>
+          <t>Owner 45, 45 Test Street, Springfield, OH, 45501, USA</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -1983,29 +1983,29 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Canada, USA</t>
+          <t>Any</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>test_dog_48@example.com</t>
+          <t>test_dog_45@example.com</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>test_dog_49</t>
+          <t>test_dog_46</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Tilly</t>
+          <t>Archie</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Owner 49, 49 Test Street, Springfield, OH, 45501, USA</t>
+          <t>Owner 46, 46 Test Street, Springfield, OH, 45501, USA</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -2020,24 +2020,24 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>test_dog_49@example.com</t>
+          <t>test_dog_46@example.com</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>test_dog_50</t>
+          <t>test_dog_47</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Bertie</t>
+          <t>Ziggy</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Owner 50, 50 Test Street, Springfield, OH, 45501, USA</t>
+          <t>Owner 47, 47 Test Street, Springfield, OH, 45501, USA</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -2052,24 +2052,24 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>test_dog_50@example.com</t>
+          <t>test_dog_47@example.com</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>test_dog_51</t>
+          <t>test_dog_48</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Nell &amp; Bertie</t>
+          <t>Biscuit</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Owner 51, 51 Test Street, Springfield, OH, 45501, USA</t>
+          <t>Owner 48, 48 Test Street, Springfield, OH, 45501, USA</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -2084,24 +2084,24 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>test_dog_51@example.com</t>
+          <t>test_dog_48@example.com</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>test_dog_52</t>
+          <t>test_dog_49</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Willow</t>
+          <t>Pippin</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Owner 52, 52 Test Street, Springfield, OH, 45501, USA</t>
+          <t>Owner 49, 49 Test Street, Springfield, OH, 45501, USA</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -2111,61 +2111,61 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Canada, USA</t>
+          <t>Any</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>test_dog_52@example.com</t>
+          <t>test_dog_49@example.com</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>test_dog_53</t>
+          <t>test_dog_49</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Hector</t>
+          <t>Otis</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Owner 53, 53 Test Street, Maple Bay, BC, V0R 1A0, Canada</t>
+          <t>Owner 49, 49 Test Street, Springfield, OH, 45501, USA</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Canada, USA</t>
+          <t>Any</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>test_dog_53@example.com</t>
+          <t>test_dog_49@example.com</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>test_dog_54</t>
+          <t>test_dog_50</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Nell</t>
+          <t>Murphy</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Owner 54, 54 Test Street, Maple Bay, BC, V0R 1A0, Canada</t>
+          <t>Owner 50, 50 Test Street, Maple Bay, BC, V0R 1A0, Canada</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -2175,29 +2175,29 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Canada, USA</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>test_dog_54@example.com</t>
+          <t>test_dog_50@example.com</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>test_dog_55</t>
+          <t>test_dog_50</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Bramble</t>
+          <t>Hector</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Owner 55, 55 Test Street, Maple Bay, BC, V0R 1A0, Canada</t>
+          <t>Owner 50, 50 Test Street, Maple Bay, BC, V0R 1A0, Canada</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -2207,29 +2207,29 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Canada, USA</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>test_dog_55@example.com</t>
+          <t>test_dog_50@example.com</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>test_dog_56</t>
+          <t>test_dog_51</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Otis</t>
+          <t>Bertie</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Owner 56, 56 Test Street, Maple Bay, BC, V0R 1A0, Canada</t>
+          <t>Owner 51, 51 Test Street, Maple Bay, BC, V0R 1A0, Canada</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -2239,29 +2239,29 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Canada, USA</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>test_dog_56@example.com</t>
+          <t>test_dog_51@example.com</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>test_dog_57</t>
+          <t>test_dog_51</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Luna</t>
+          <t>Bramble</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Owner 57, 57 Test Street, Maple Bay, BC, V0R 1A0, Canada</t>
+          <t>Owner 51, 51 Test Street, Maple Bay, BC, V0R 1A0, Canada</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -2271,29 +2271,29 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Canada, USA</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>test_dog_57@example.com</t>
+          <t>test_dog_51@example.com</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>test_dog_58</t>
+          <t>test_dog_52</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Bertie</t>
+          <t>Willow</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Owner 58, 58 Test Street, Maple Bay, BC, V0R 1A0, Canada</t>
+          <t>Owner 52, 52 Test Street, Maple Bay, BC, V0R 1A0, Canada</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -2303,61 +2303,61 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Canada, USA</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>test_dog_58@example.com</t>
+          <t>test_dog_52@example.com</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>test_dog_59</t>
+          <t>test_dog_53</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Tilly</t>
+          <t>Rolo</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Owner 59, 59 Test Street, Maple Bay, BC, V0R 1A0, Canada</t>
+          <t>Owner 53, 53 Test Street, Kangaroo Flat VIC, 3555, Australia</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Canada, USA</t>
+          <t>Any</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>test_dog_59@example.com</t>
+          <t>test_dog_53@example.com</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>test_dog_60</t>
+          <t>test_dog_54</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Nell</t>
+          <t>Clover</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Owner 60, 60 Test Street, Kangaroo Flat VIC, 3555, Australia</t>
+          <t>Owner 54, 54 Test Street, Kangaroo Flat VIC, 3555, Australia</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -2367,29 +2367,29 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Any</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>test_dog_60@example.com</t>
+          <t>test_dog_54@example.com</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>test_dog_61</t>
+          <t>test_dog_55</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Nell</t>
+          <t>Bertie</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Owner 61, 61 Test Street, Kangaroo Flat VIC, 3555, Australia</t>
+          <t>Owner 55, 55 Test Street, Kangaroo Flat VIC, 3555, Australia</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -2399,29 +2399,29 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Any</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>test_dog_61@example.com</t>
+          <t>test_dog_55@example.com</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>test_dog_62</t>
+          <t>test_dog_56</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Luna &amp; Tilly</t>
+          <t>Nell</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Owner 62, 62 Test Street, Kangaroo Flat VIC, 3555, Australia</t>
+          <t>Owner 56, 56 Test Street, Kangaroo Flat VIC, 3555, Australia</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -2431,29 +2431,29 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Any</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>test_dog_62@example.com</t>
+          <t>test_dog_56@example.com</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>test_dog_63</t>
+          <t>test_dog_57</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Otis</t>
+          <t>Pippin</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Owner 63, 63 Test Street, Kangaroo Flat VIC, 3555, Australia</t>
+          <t>Owner 57, 57 Test Street, Kangaroo Flat VIC, 3555, Australia</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -2468,24 +2468,24 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>test_dog_63@example.com</t>
+          <t>test_dog_57@example.com</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>test_dog_64</t>
+          <t>test_dog_58</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Bertie</t>
+          <t>Tilly</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Owner 64, 64 Test Street, Kangaroo Flat VIC, 3555, Australia</t>
+          <t>Owner 58, 58 Test Street, Kangaroo Flat VIC, 3555, Australia</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -2500,24 +2500,24 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>test_dog_64@example.com</t>
+          <t>test_dog_58@example.com</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>test_dog_65</t>
+          <t>test_dog_59</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Rolo</t>
+          <t>Pippin</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Owner 65, 65 Test Street, Kangaroo Flat VIC, 3555, Australia</t>
+          <t>Owner 59, 59 Test Street, Kangaroo Flat VIC, 3555, Australia</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -2527,19 +2527,19 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Any</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>test_dog_65@example.com</t>
+          <t>test_dog_59@example.com</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>test_dog_66</t>
+          <t>test_dog_60</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2549,204 +2549,204 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Owner 66, 66 Test Street, Kangaroo Flat VIC, 3555, Australia</t>
+          <t>Owner 60, 60 Test Street, Reykjavik, 101, Iceland</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Iceland</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Iceland</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>test_dog_66@example.com</t>
+          <t>test_dog_60@example.com</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>test_dog_67</t>
+          <t>test_dog_61</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Tilly</t>
+          <t>Mabel</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Owner 67, 67 Test Street, Kangaroo Flat VIC, 3555, Australia</t>
+          <t>Owner 61, 61 Test Street, Reykjavik, 101, Iceland</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Iceland</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Any</t>
+          <t>Iceland</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>test_dog_67@example.com</t>
+          <t>test_dog_61@example.com</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>test_dog_68</t>
+          <t>test_dog_62</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Bramble &amp; Archie</t>
+          <t>Willow</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Owner 68, 68 Test Street, Reykjavik, 101, Iceland</t>
+          <t>Owner 62, 62 Test Street, Musterstadt, 12345, Germany</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Iceland</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Iceland</t>
+          <t>EU</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>test_dog_68@example.com</t>
+          <t>test_dog_62@example.com</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>test_dog_69</t>
+          <t>test_dog_63</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Rolo</t>
+          <t>Ziggy</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Owner 69, 69 Test Street, Reykjavik, 101, Iceland</t>
+          <t>Owner 63, 63 Test Street, Musterstadt, 12345, Germany</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Iceland</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Any</t>
+          <t>EU</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>test_dog_69@example.com</t>
+          <t>test_dog_63@example.com</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>test_dog_70</t>
+          <t>test_dog_64</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Pippin &amp; Murphy</t>
+          <t>Otis</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Owner 70, 70 Test Street, Musterstadt, 12345, Germany</t>
+          <t>Owner 64, 64 Test Street, Voorbeeld, 1234 AB, The Netherlands</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>The Netherlands</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>Any</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>test_dog_70@example.com</t>
+          <t>test_dog_64@example.com</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>test_dog_71</t>
+          <t>test_dog_65</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Pippin</t>
+          <t>Fudge</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Owner 71, 71 Test Street, Musterstadt, 12345, Germany</t>
+          <t>Owner 65, 65 Test Street, Voorbeeld, 1234 AB, The Netherlands</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>The Netherlands</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>Any</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>test_dog_71@example.com</t>
+          <t>test_dog_65@example.com</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>test_dog_72</t>
+          <t>test_dog_66</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Tilly</t>
+          <t>Archie</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Owner 72, 72 Test Street, Voorbeeld, 1234 AB, The Netherlands</t>
+          <t>Owner 66, 66 Test Street, Exempleville, 75000, France</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>The Netherlands</t>
+          <t>France</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -2756,29 +2756,29 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>test_dog_72@example.com</t>
+          <t>test_dog_66@example.com</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>test_dog_73</t>
+          <t>test_dog_67</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Pippin &amp; Biscuit</t>
+          <t>Ziggy</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Owner 73, 73 Test Street, Voorbeeld, 1234 AB, The Netherlands</t>
+          <t>Owner 67, 67 Test Street, Exempleville, 75000, France</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>The Netherlands</t>
+          <t>France</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -2788,61 +2788,61 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>test_dog_73@example.com</t>
+          <t>test_dog_67@example.com</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>test_dog_74</t>
+          <t>test_dog_68</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Pippin</t>
+          <t>Daisy</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Owner 74, 74 Test Street, Exempleville, 75000, France</t>
+          <t>Owner 68, 68 Test Street, Esempio, 00100, Italy</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>Any</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>test_dog_74@example.com</t>
+          <t>test_dog_68@example.com</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>test_dog_75</t>
+          <t>test_dog_69</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Otis &amp; Otis</t>
+          <t>Daisy</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Owner 75, 75 Test Street, Exempleville, 75000, France</t>
+          <t>Owner 69, 69 Test Street, Esempio, 00100, Italy</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -2852,61 +2852,61 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>test_dog_75@example.com</t>
+          <t>test_dog_69@example.com</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>test_dog_76</t>
+          <t>test_dog_70</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Luna</t>
+          <t>Hector</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Owner 76, 76 Test Street, Esempio, 00100, Italy</t>
+          <t>Owner 70, 70 Test Street, Primjer, 10000, Croatia</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Croatia</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Any</t>
+          <t>EU</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>test_dog_76@example.com</t>
+          <t>test_dog_70@example.com</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>test_dog_77</t>
+          <t>test_dog_71</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Poppy</t>
+          <t>Archie</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Owner 77, 77 Test Street, Esempio, 00100, Italy</t>
+          <t>Owner 71, 71 Test Street, Primjer, 10000, Croatia</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Croatia</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -2916,103 +2916,39 @@
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>test_dog_77@example.com</t>
+          <t>test_dog_71@example.com</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>test_dog_78</t>
+          <t>test_dog_72</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Nell</t>
+          <t>Hector</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Owner 78, 78 Test Street, Primjer, 10000, Croatia</t>
+          <t>Owner 72, 72 Test Street, Tokyo, 100-0001, Japan</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Croatia</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>Any</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>test_dog_78@example.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" t="inlineStr">
-        <is>
-          <t>test_dog_79</t>
-        </is>
-      </c>
-      <c r="B80" t="inlineStr">
-        <is>
-          <t>Poppy</t>
-        </is>
-      </c>
-      <c r="C80" t="inlineStr">
-        <is>
-          <t>Owner 79, 79 Test Street, Primjer, 10000, Croatia</t>
-        </is>
-      </c>
-      <c r="D80" t="inlineStr">
-        <is>
-          <t>Croatia</t>
-        </is>
-      </c>
-      <c r="E80" t="inlineStr">
-        <is>
-          <t>EU</t>
-        </is>
-      </c>
-      <c r="F80" t="inlineStr">
-        <is>
-          <t>test_dog_79@example.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" t="inlineStr">
-        <is>
-          <t>test_dog_80</t>
-        </is>
-      </c>
-      <c r="B81" t="inlineStr">
-        <is>
-          <t>Pippin</t>
-        </is>
-      </c>
-      <c r="C81" t="inlineStr">
-        <is>
-          <t>Owner 80, 80 Test Street, Tokyo, 100-0001, Japan</t>
-        </is>
-      </c>
-      <c r="D81" t="inlineStr">
-        <is>
-          <t>Japan</t>
-        </is>
-      </c>
-      <c r="E81" t="inlineStr">
-        <is>
-          <t>Any</t>
-        </is>
-      </c>
-      <c r="F81" t="inlineStr">
-        <is>
-          <t>test_dog_80@example.com</t>
+          <t>test_dog_72@example.com</t>
         </is>
       </c>
     </row>

</xml_diff>